<commit_message>
data(week 19): refresh inventory snapshots
Re-saved per-brand Inventory Snapshot.xlsx for Audio_Array, Nexlev,
Tonor, White_Mulberry — minor size changes from upstream re-export.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/inventory/Week 19/Audio_Array/Inventory Snapshot.xlsx
+++ b/data/raw/inventory/Week 19/Audio_Array/Inventory Snapshot.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 19\Audio_Array\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{601B3C29-D3D2-415B-9556-1907EA39FEFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DCDC3F0-0C80-4C14-B878-B82612875ACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D49B0F4C-5F9E-467E-8AD9-9E638F42404F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3056" uniqueCount="636">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3311" uniqueCount="680">
   <si>
     <t>SKU</t>
   </si>
@@ -1945,6 +1945,138 @@
   </si>
   <si>
     <t>PB-08 (AM-C1 + AI-04)</t>
+  </si>
+  <si>
+    <t>Pipeline</t>
+  </si>
+  <si>
+    <t>FBA80109</t>
+  </si>
+  <si>
+    <t>FBA80110</t>
+  </si>
+  <si>
+    <t>FBA80119</t>
+  </si>
+  <si>
+    <t>FBA80120</t>
+  </si>
+  <si>
+    <t>FBA80121</t>
+  </si>
+  <si>
+    <t>FBA80122</t>
+  </si>
+  <si>
+    <t>FBA80123</t>
+  </si>
+  <si>
+    <t>FBA80124</t>
+  </si>
+  <si>
+    <t>FBA80125</t>
+  </si>
+  <si>
+    <t>FBA80126</t>
+  </si>
+  <si>
+    <t>FBA80129</t>
+  </si>
+  <si>
+    <t>FBA80130</t>
+  </si>
+  <si>
+    <t>FBA80131</t>
+  </si>
+  <si>
+    <t>FBA80132</t>
+  </si>
+  <si>
+    <t>FBA80133</t>
+  </si>
+  <si>
+    <t>FBA80134</t>
+  </si>
+  <si>
+    <t>FBA80135</t>
+  </si>
+  <si>
+    <t>FBA80136</t>
+  </si>
+  <si>
+    <t>FBA80137</t>
+  </si>
+  <si>
+    <t>FBA80138</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AC-6XL	</t>
+  </si>
+  <si>
+    <t>AM-S6</t>
+  </si>
+  <si>
+    <t>M5</t>
+  </si>
+  <si>
+    <t>X5</t>
+  </si>
+  <si>
+    <t>AM-C53</t>
+  </si>
+  <si>
+    <t>AM-C54</t>
+  </si>
+  <si>
+    <t>AM-C55</t>
+  </si>
+  <si>
+    <t>AM-C56</t>
+  </si>
+  <si>
+    <t>AM-W25</t>
+  </si>
+  <si>
+    <t>AA-26 Pro</t>
+  </si>
+  <si>
+    <t>AA-28</t>
+  </si>
+  <si>
+    <t>AA-29</t>
+  </si>
+  <si>
+    <t>HP4</t>
+  </si>
+  <si>
+    <t>HPA1400</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>PRE103</t>
+  </si>
+  <si>
+    <t>DI20</t>
+  </si>
+  <si>
+    <t>AC1</t>
+  </si>
+  <si>
+    <t>IS-2</t>
+  </si>
+  <si>
+    <t>IS-3</t>
+  </si>
+  <si>
+    <t>P7</t>
+  </si>
+  <si>
+    <t>MS155</t>
+  </si>
+  <si>
+    <t>Open Order</t>
   </si>
 </sst>
 </file>
@@ -2071,7 +2203,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2107,13 +2239,110 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{697FC575-8A7C-4715-A8F0-2950C62D8576}"/>
     <cellStyle name="Normal 6" xfId="1" xr:uid="{E5F241CE-C0FC-4730-81C9-F1901EB82A3C}"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="18">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2534,7 +2763,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}">
-  <dimension ref="A1:L610"/>
+  <dimension ref="A1:L665"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
@@ -14803,29 +15032,1082 @@
       </c>
       <c r="K610" s="10"/>
     </row>
+    <row r="611" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A611" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B611" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="C611" t="s">
+        <v>477</v>
+      </c>
+      <c r="D611" s="13" t="s">
+        <v>431</v>
+      </c>
+      <c r="I611" s="1">
+        <v>1035</v>
+      </c>
+      <c r="J611" s="1" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="612" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A612" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B612" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="C612" t="s">
+        <v>477</v>
+      </c>
+      <c r="D612" s="13" t="s">
+        <v>432</v>
+      </c>
+      <c r="I612" s="1">
+        <v>768</v>
+      </c>
+      <c r="J612" s="1" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="613" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A613" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B613" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="C613" t="s">
+        <v>477</v>
+      </c>
+      <c r="D613" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="I613" s="1">
+        <v>1008</v>
+      </c>
+      <c r="J613" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="614" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A614" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B614" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C614" t="s">
+        <v>477</v>
+      </c>
+      <c r="D614" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="I614" s="1">
+        <v>3000</v>
+      </c>
+      <c r="J614" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="615" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A615" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B615" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C615" t="s">
+        <v>477</v>
+      </c>
+      <c r="D615" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="I615" s="1">
+        <v>1000</v>
+      </c>
+      <c r="J615" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="616" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A616" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B616" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="C616" t="s">
+        <v>477</v>
+      </c>
+      <c r="D616" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="I616" s="1">
+        <v>1000</v>
+      </c>
+      <c r="J616" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="617" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A617" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B617" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C617" t="s">
+        <v>477</v>
+      </c>
+      <c r="D617" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="I617" s="1">
+        <v>3000</v>
+      </c>
+      <c r="J617" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="618" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A618" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B618" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="C618" t="s">
+        <v>477</v>
+      </c>
+      <c r="D618" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="I618" s="1">
+        <v>1496</v>
+      </c>
+      <c r="J618" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="619" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A619" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B619" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C619" t="s">
+        <v>477</v>
+      </c>
+      <c r="D619" s="1" t="s">
+        <v>657</v>
+      </c>
+      <c r="I619" s="1">
+        <v>2000</v>
+      </c>
+      <c r="J619" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="620" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A620" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B620" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C620" t="s">
+        <v>477</v>
+      </c>
+      <c r="D620" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="I620" s="1">
+        <v>501</v>
+      </c>
+      <c r="J620" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="621" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A621" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B621" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="C621" t="s">
+        <v>477</v>
+      </c>
+      <c r="D621" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="I621" s="1">
+        <v>504</v>
+      </c>
+      <c r="J621" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="622" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A622" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B622" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C622" t="s">
+        <v>477</v>
+      </c>
+      <c r="D622" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="I622" s="1">
+        <v>504</v>
+      </c>
+      <c r="J622" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="623" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A623" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B623" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C623" t="s">
+        <v>477</v>
+      </c>
+      <c r="D623" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="I623" s="1">
+        <v>201</v>
+      </c>
+      <c r="J623" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="624" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A624" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B624" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="C624" t="s">
+        <v>477</v>
+      </c>
+      <c r="D624" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="I624" s="1">
+        <v>512</v>
+      </c>
+      <c r="J624" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="625" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A625" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B625" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="C625" t="s">
+        <v>477</v>
+      </c>
+      <c r="D625" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="I625" s="1">
+        <v>1000</v>
+      </c>
+      <c r="J625" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="626" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A626" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B626" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C626" t="s">
+        <v>477</v>
+      </c>
+      <c r="D626" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="I626" s="1">
+        <v>480</v>
+      </c>
+      <c r="J626" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="627" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A627" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B627" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="C627" t="s">
+        <v>477</v>
+      </c>
+      <c r="D627" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="I627" s="1">
+        <v>504</v>
+      </c>
+      <c r="J627" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="628" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A628" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B628" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="C628" t="s">
+        <v>477</v>
+      </c>
+      <c r="D628" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="I628" s="1">
+        <v>1000</v>
+      </c>
+      <c r="J628" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="629" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A629" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B629" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C629" t="s">
+        <v>477</v>
+      </c>
+      <c r="D629" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="I629" s="1">
+        <v>500</v>
+      </c>
+      <c r="J629" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="630" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A630" s="1" t="s">
+        <v>577</v>
+      </c>
+      <c r="B630" s="1" t="s">
+        <v>578</v>
+      </c>
+      <c r="C630" t="s">
+        <v>477</v>
+      </c>
+      <c r="D630" s="1" t="s">
+        <v>619</v>
+      </c>
+      <c r="I630" s="1">
+        <v>20</v>
+      </c>
+      <c r="J630" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="631" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A631" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B631" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C631" t="s">
+        <v>477</v>
+      </c>
+      <c r="D631" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="I631" s="1">
+        <v>504</v>
+      </c>
+      <c r="J631" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="632" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A632" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B632" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="C632" t="s">
+        <v>477</v>
+      </c>
+      <c r="D632" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="I632" s="1">
+        <v>2000</v>
+      </c>
+      <c r="J632" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="633" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A633" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B633" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="C633" t="s">
+        <v>477</v>
+      </c>
+      <c r="D633" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="I633" s="1">
+        <v>990</v>
+      </c>
+      <c r="J633" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="634" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A634" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B634" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="C634" t="s">
+        <v>477</v>
+      </c>
+      <c r="D634" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="I634" s="1">
+        <v>744</v>
+      </c>
+      <c r="J634" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="635" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A635" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B635" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="C635" t="s">
+        <v>477</v>
+      </c>
+      <c r="D635" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="I635" s="1">
+        <v>500</v>
+      </c>
+      <c r="J635" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="636" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A636" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B636" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="C636" t="s">
+        <v>477</v>
+      </c>
+      <c r="D636" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="I636" s="1">
+        <v>1300</v>
+      </c>
+      <c r="J636" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="637" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A637" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B637" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="C637" t="s">
+        <v>477</v>
+      </c>
+      <c r="D637" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="I637" s="1">
+        <v>600</v>
+      </c>
+      <c r="J637" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="638" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A638" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B638" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="C638" t="s">
+        <v>477</v>
+      </c>
+      <c r="D638" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="I638" s="1">
+        <v>140</v>
+      </c>
+      <c r="J638" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="639" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A639" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B639" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="C639" t="s">
+        <v>477</v>
+      </c>
+      <c r="D639" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="I639" s="1">
+        <v>150</v>
+      </c>
+      <c r="J639" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="640" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A640" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B640" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="C640" t="s">
+        <v>477</v>
+      </c>
+      <c r="D640" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="I640" s="1">
+        <v>400</v>
+      </c>
+      <c r="J640" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="641" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A641" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B641" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="C641" t="s">
+        <v>477</v>
+      </c>
+      <c r="D641" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="I641" s="1">
+        <v>200</v>
+      </c>
+      <c r="J641" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="642" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A642" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B642" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="C642" t="s">
+        <v>477</v>
+      </c>
+      <c r="D642" s="1" t="s">
+        <v>658</v>
+      </c>
+      <c r="I642" s="1">
+        <v>50</v>
+      </c>
+      <c r="J642" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="643" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A643" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B643" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="C643" t="s">
+        <v>477</v>
+      </c>
+      <c r="D643" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="I643" s="1">
+        <v>1004</v>
+      </c>
+      <c r="J643" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="644" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A644" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B644" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="C644" t="s">
+        <v>477</v>
+      </c>
+      <c r="D644" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="I644" s="1">
+        <v>300</v>
+      </c>
+      <c r="J644" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="645" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A645" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B645" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="C645" t="s">
+        <v>477</v>
+      </c>
+      <c r="D645" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="I645" s="1">
+        <v>400</v>
+      </c>
+      <c r="J645" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="646" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A646" s="1" t="s">
+        <v>637</v>
+      </c>
+      <c r="C646" t="s">
+        <v>477</v>
+      </c>
+      <c r="D646" s="1" t="s">
+        <v>659</v>
+      </c>
+      <c r="I646" s="1">
+        <v>20</v>
+      </c>
+      <c r="J646" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="647" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A647" s="1" t="s">
+        <v>638</v>
+      </c>
+      <c r="C647" t="s">
+        <v>477</v>
+      </c>
+      <c r="D647" s="1" t="s">
+        <v>660</v>
+      </c>
+      <c r="I647" s="1">
+        <v>20</v>
+      </c>
+      <c r="J647" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="648" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A648" s="1" t="s">
+        <v>639</v>
+      </c>
+      <c r="C648" t="s">
+        <v>477</v>
+      </c>
+      <c r="D648" s="1" t="s">
+        <v>661</v>
+      </c>
+      <c r="I648" s="1">
+        <v>510</v>
+      </c>
+      <c r="J648" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="649" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A649" s="1" t="s">
+        <v>640</v>
+      </c>
+      <c r="C649" t="s">
+        <v>477</v>
+      </c>
+      <c r="D649" s="1" t="s">
+        <v>662</v>
+      </c>
+      <c r="I649" s="1">
+        <v>510</v>
+      </c>
+      <c r="J649" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="650" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A650" s="1" t="s">
+        <v>641</v>
+      </c>
+      <c r="C650" t="s">
+        <v>477</v>
+      </c>
+      <c r="D650" s="1" t="s">
+        <v>663</v>
+      </c>
+      <c r="I650" s="1">
+        <v>500</v>
+      </c>
+      <c r="J650" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="651" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A651" s="1" t="s">
+        <v>642</v>
+      </c>
+      <c r="C651" t="s">
+        <v>477</v>
+      </c>
+      <c r="D651" s="1" t="s">
+        <v>664</v>
+      </c>
+      <c r="I651" s="1">
+        <v>504</v>
+      </c>
+      <c r="J651" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="652" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A652" s="1" t="s">
+        <v>643</v>
+      </c>
+      <c r="C652" t="s">
+        <v>477</v>
+      </c>
+      <c r="D652" s="1" t="s">
+        <v>665</v>
+      </c>
+      <c r="I652" s="1">
+        <v>60</v>
+      </c>
+      <c r="J652" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="653" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A653" s="1" t="s">
+        <v>644</v>
+      </c>
+      <c r="C653" t="s">
+        <v>477</v>
+      </c>
+      <c r="D653" s="1" t="s">
+        <v>666</v>
+      </c>
+      <c r="I653" s="1">
+        <v>1000</v>
+      </c>
+      <c r="J653" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="654" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A654" s="1" t="s">
+        <v>645</v>
+      </c>
+      <c r="C654" t="s">
+        <v>477</v>
+      </c>
+      <c r="D654" s="1" t="s">
+        <v>667</v>
+      </c>
+      <c r="I654" s="1">
+        <v>100</v>
+      </c>
+      <c r="J654" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="655" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A655" s="1" t="s">
+        <v>646</v>
+      </c>
+      <c r="C655" t="s">
+        <v>477</v>
+      </c>
+      <c r="D655" s="1" t="s">
+        <v>668</v>
+      </c>
+      <c r="I655" s="1">
+        <v>100</v>
+      </c>
+      <c r="J655" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="656" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A656" s="1" t="s">
+        <v>647</v>
+      </c>
+      <c r="C656" t="s">
+        <v>477</v>
+      </c>
+      <c r="D656" s="1" t="s">
+        <v>669</v>
+      </c>
+      <c r="I656" s="1">
+        <v>20</v>
+      </c>
+      <c r="J656" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="657" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A657" s="1" t="s">
+        <v>648</v>
+      </c>
+      <c r="C657" t="s">
+        <v>477</v>
+      </c>
+      <c r="D657" s="1" t="s">
+        <v>670</v>
+      </c>
+      <c r="I657" s="1">
+        <v>20</v>
+      </c>
+      <c r="J657" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="658" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A658" s="1" t="s">
+        <v>649</v>
+      </c>
+      <c r="C658" t="s">
+        <v>477</v>
+      </c>
+      <c r="D658" s="1" t="s">
+        <v>671</v>
+      </c>
+      <c r="I658" s="1">
+        <v>20</v>
+      </c>
+      <c r="J658" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="659" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A659" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="C659" t="s">
+        <v>477</v>
+      </c>
+      <c r="D659" s="1" t="s">
+        <v>672</v>
+      </c>
+      <c r="I659" s="1">
+        <v>20</v>
+      </c>
+      <c r="J659" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="660" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A660" s="1" t="s">
+        <v>651</v>
+      </c>
+      <c r="C660" t="s">
+        <v>477</v>
+      </c>
+      <c r="D660" s="1" t="s">
+        <v>673</v>
+      </c>
+      <c r="I660" s="1">
+        <v>20</v>
+      </c>
+      <c r="J660" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="661" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A661" s="1" t="s">
+        <v>652</v>
+      </c>
+      <c r="C661" t="s">
+        <v>477</v>
+      </c>
+      <c r="D661" s="1" t="s">
+        <v>674</v>
+      </c>
+      <c r="I661" s="1">
+        <v>20</v>
+      </c>
+      <c r="J661" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="662" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A662" s="1" t="s">
+        <v>653</v>
+      </c>
+      <c r="C662" t="s">
+        <v>477</v>
+      </c>
+      <c r="D662" s="1" t="s">
+        <v>675</v>
+      </c>
+      <c r="I662" s="1">
+        <v>20</v>
+      </c>
+      <c r="J662" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="663" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A663" s="1" t="s">
+        <v>654</v>
+      </c>
+      <c r="C663" t="s">
+        <v>477</v>
+      </c>
+      <c r="D663" s="1" t="s">
+        <v>676</v>
+      </c>
+      <c r="I663" s="1">
+        <v>20</v>
+      </c>
+      <c r="J663" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="664" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A664" s="1" t="s">
+        <v>655</v>
+      </c>
+      <c r="C664" t="s">
+        <v>477</v>
+      </c>
+      <c r="D664" s="1" t="s">
+        <v>677</v>
+      </c>
+      <c r="I664" s="1">
+        <v>20</v>
+      </c>
+      <c r="J664" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="665" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A665" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="C665" t="s">
+        <v>477</v>
+      </c>
+      <c r="D665" s="1" t="s">
+        <v>678</v>
+      </c>
+      <c r="I665" s="1">
+        <v>20</v>
+      </c>
+      <c r="J665" s="1" t="s">
+        <v>679</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L610" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}"/>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="A348:A507">
+    <cfRule type="duplicateValues" dxfId="17" priority="1602"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A456">
+    <cfRule type="duplicateValues" dxfId="16" priority="1600"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="duplicateValues" dxfId="8" priority="1353"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="1362"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:H1">
-    <cfRule type="duplicateValues" dxfId="7" priority="1564"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="1565" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="1573"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="1574" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="duplicateValues" dxfId="5" priority="1351"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="1352" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="1360"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="1361" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:L1">
-    <cfRule type="duplicateValues" dxfId="3" priority="1349"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="1350" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="1358"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="1359" stopIfTrue="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A456">
-    <cfRule type="duplicateValues" dxfId="1" priority="1591"/>
+  <conditionalFormatting sqref="A611:A612">
+    <cfRule type="duplicateValues" dxfId="8" priority="9"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A348:A507">
-    <cfRule type="duplicateValues" dxfId="0" priority="1593"/>
+  <conditionalFormatting sqref="D611:D612">
+    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="7" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="8" stopIfTrue="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>